<commit_message>
Updated Part Selection Doc.
New components added and previous ones have been updated according to the new circuit design guidelines.
</commit_message>
<xml_diff>
--- a/Documents/Part Selection.xlsx
+++ b/Documents/Part Selection.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\SaleemD-CustomProduct\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{720D0AF8-62F6-4B43-A283-FAA45649EDA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE4024D9-FBCE-416E-BC82-DBE2F5DA7C1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{485F4B6F-F421-4A15-A4EA-AEFC940F358A}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="51">
   <si>
     <t>Buck regulator</t>
   </si>
@@ -66,22 +66,118 @@
     <t>Part number</t>
   </si>
   <si>
-    <t>XL1583E1</t>
-  </si>
-  <si>
     <t>STM32F030F4P6</t>
   </si>
   <si>
-    <t>AP22814AW5-7</t>
-  </si>
-  <si>
-    <t>B3B-XH-A(LF)(SN)</t>
-  </si>
-  <si>
-    <t>Mouser</t>
-  </si>
-  <si>
-    <t>SN74LV1T34DBVR</t>
+    <t>For 12A and 6A</t>
+  </si>
+  <si>
+    <t>3.3V regulator</t>
+  </si>
+  <si>
+    <t>NCP1117LPST33T3G</t>
+  </si>
+  <si>
+    <t>Terminal blocks</t>
+  </si>
+  <si>
+    <t>WJ126V-5.0-6P</t>
+  </si>
+  <si>
+    <t>Ferrite bead</t>
+  </si>
+  <si>
+    <t>SBM1608G601GSP</t>
+  </si>
+  <si>
+    <t>Crystal</t>
+  </si>
+  <si>
+    <t>X1A000061002100</t>
+  </si>
+  <si>
+    <t>32.768KHz</t>
+  </si>
+  <si>
+    <t>8MHz</t>
+  </si>
+  <si>
+    <t>XXDCCLNANF-8.000000MHZ</t>
+  </si>
+  <si>
+    <t>Capacitors</t>
+  </si>
+  <si>
+    <t>any capacitors with 0603 package</t>
+  </si>
+  <si>
+    <t>100nF/25V</t>
+  </si>
+  <si>
+    <t>1uF/25V</t>
+  </si>
+  <si>
+    <t>4.7uF/25V</t>
+  </si>
+  <si>
+    <t>10nF/25V</t>
+  </si>
+  <si>
+    <t>B3U-1000P</t>
+  </si>
+  <si>
+    <t>Aliexpress</t>
+  </si>
+  <si>
+    <t>Resistor</t>
+  </si>
+  <si>
+    <t>640456-3</t>
+  </si>
+  <si>
+    <t>Transistor</t>
+  </si>
+  <si>
+    <t>IRF530SPBF</t>
+  </si>
+  <si>
+    <t>RC2512JK-07100RL</t>
+  </si>
+  <si>
+    <t>100R</t>
+  </si>
+  <si>
+    <t>1K/0603</t>
+  </si>
+  <si>
+    <t>Tactile switch</t>
+  </si>
+  <si>
+    <t>6 pin header for programming</t>
+  </si>
+  <si>
+    <t>SLG59M1470V</t>
+  </si>
+  <si>
+    <t>DigiKey</t>
+  </si>
+  <si>
+    <t>52.5K</t>
+  </si>
+  <si>
+    <t>10K</t>
+  </si>
+  <si>
+    <t>Inductor</t>
+  </si>
+  <si>
+    <t>Not available on LCSC</t>
+  </si>
+  <si>
+    <t>ASPI-0530LR-3R3M-T2</t>
+  </si>
+  <si>
+    <t>SN74LV07APWR</t>
   </si>
 </sst>
 </file>
@@ -170,7 +266,10 @@
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="8">
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -194,7 +293,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="Table Style 1" pivot="0" count="1" xr9:uid="{353EA788-3CED-4D42-8479-F2529B036161}"/>
+    <tableStyle name="Table Style 1" pivot="0" count="0" xr9:uid="{353EA788-3CED-4D42-8479-F2529B036161}"/>
   </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -208,13 +307,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{87DDCAFF-B5E3-4BC3-8443-CED7736DCCFF}" name="Table5" displayName="Table5" ref="A3:E7" headerRowCount="0" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
-  <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{00E16EC1-2113-4612-8235-E9DF3502C29A}" name="Column1" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{794E69B8-0E31-4F55-BCF0-8AC80C796848}" name="Column2" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{00D1FB53-C6BA-4B12-B3E8-2B17B495AC02}" name="Column3" dataDxfId="4" headerRowCellStyle="Hyperlink" dataCellStyle="Hyperlink"/>
-    <tableColumn id="4" xr3:uid="{7B92CE0D-AFEA-4157-A8B1-040122A40A11}" name="Column4" dataDxfId="3" headerRowCellStyle="Hyperlink"/>
-    <tableColumn id="5" xr3:uid="{8E2C99BA-66A9-4525-89E5-660A240E0F77}" name="Column5" dataDxfId="2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{87DDCAFF-B5E3-4BC3-8443-CED7736DCCFF}" name="Table5" displayName="Table5" ref="A3:F24" headerRowCount="0" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{00E16EC1-2113-4612-8235-E9DF3502C29A}" name="Column1" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{794E69B8-0E31-4F55-BCF0-8AC80C796848}" name="Column2" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{68043DCE-DFEC-47BE-8E96-4391C9421392}" name="Column6" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{00D1FB53-C6BA-4B12-B3E8-2B17B495AC02}" name="Column3" dataDxfId="3" headerRowCellStyle="Hyperlink" dataCellStyle="Hyperlink"/>
+    <tableColumn id="4" xr3:uid="{7B92CE0D-AFEA-4157-A8B1-040122A40A11}" name="Column4" dataDxfId="2" headerRowCellStyle="Hyperlink"/>
+    <tableColumn id="5" xr3:uid="{8E2C99BA-66A9-4525-89E5-660A240E0F77}" name="Column5" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -517,120 +617,364 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83A19A4C-3AFB-4FAF-A2B0-E08575584D2A}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
     <col min="2" max="2" width="27" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="13.140625" customWidth="1"/>
-    <col min="5" max="5" width="32.85546875" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="13.140625" customWidth="1"/>
+    <col min="6" max="6" width="32.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="C1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="2"/>
+      <c r="D2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>2</v>
-      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
       <c r="D3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="3"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E3" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D4" s="3"/>
+        <v>13</v>
+      </c>
+      <c r="C4" s="3"/>
+      <c r="D4" s="4" t="s">
+        <v>2</v>
+      </c>
       <c r="E4" s="3"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F4" s="3"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D5" s="3"/>
+        <v>50</v>
+      </c>
+      <c r="C5" s="3"/>
+      <c r="D5" s="4" t="s">
+        <v>2</v>
+      </c>
       <c r="E5" s="3"/>
-    </row>
-    <row r="6" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="F5" s="3"/>
+    </row>
+    <row r="6" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="3"/>
-      <c r="E6" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" s="3"/>
+      <c r="D6" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E6" s="3"/>
+      <c r="F6" s="5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" s="3"/>
+      <c r="D7" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F8" s="3"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="3"/>
+      <c r="D9" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" s="4"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="3"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D11" s="4"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D12" s="4"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="3"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" s="4"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C14" s="3"/>
+      <c r="D14" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F14" s="3"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C15" s="3"/>
+      <c r="D15" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" s="3"/>
+      <c r="D16" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="3"/>
+      <c r="B18" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="3"/>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D20" s="4"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="3"/>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D21" s="4"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="3"/>
+      <c r="B22" s="3"/>
+      <c r="C22" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D22" s="4"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+    </row>
+    <row r="23" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3" t="s">
+        <v>48</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C3" r:id="rId1" xr:uid="{E44A0F55-6434-40A2-9C4E-0AA902DB5CB4}"/>
-    <hyperlink ref="D3" r:id="rId2" xr:uid="{1D03B396-EADA-40AF-A9ED-3558493F76A6}"/>
-    <hyperlink ref="C4" r:id="rId3" xr:uid="{F2B0A6EA-D78B-4B49-A962-6660BB86D401}"/>
-    <hyperlink ref="C6" r:id="rId4" xr:uid="{CF0FAEAF-11DE-4D98-9F48-8E5CFAE8B0A4}"/>
-    <hyperlink ref="C7" r:id="rId5" xr:uid="{D6CB9D3C-A827-41E9-9096-EE0CBEA4F8E9}"/>
-    <hyperlink ref="C5" r:id="rId6" xr:uid="{8672460E-B561-4B8C-B0F5-C3EC9A14256B}"/>
+    <hyperlink ref="D4" r:id="rId1" xr:uid="{F2B0A6EA-D78B-4B49-A962-6660BB86D401}"/>
+    <hyperlink ref="D5" r:id="rId2" xr:uid="{8672460E-B561-4B8C-B0F5-C3EC9A14256B}"/>
+    <hyperlink ref="D3" r:id="rId3" xr:uid="{3C7C5C37-32E7-4651-B908-0D6E51211522}"/>
+    <hyperlink ref="E3" r:id="rId4" xr:uid="{205B6E06-8222-456E-9A56-815CDA53CF40}"/>
+    <hyperlink ref="D8" r:id="rId5" xr:uid="{5D79376F-C20A-49E7-896F-E2C395EC5A8D}"/>
+    <hyperlink ref="E8" r:id="rId6" xr:uid="{5F52FA42-411A-464D-B088-9E03F4F7BBFB}"/>
+    <hyperlink ref="D9" r:id="rId7" xr:uid="{14C870E9-3CF6-4DA7-B5DF-BAD6E02E5C17}"/>
+    <hyperlink ref="D16" r:id="rId8" xr:uid="{9039FBC5-A2EE-4B40-B3AF-721FC5523F1B}"/>
+    <hyperlink ref="D17" r:id="rId9" xr:uid="{87CAEA90-6EC4-4C15-8ABD-7A412E31C0F3}"/>
+    <hyperlink ref="D18" r:id="rId10" xr:uid="{F8BC75E1-2481-4659-986A-03D7D6A3DB5A}"/>
+    <hyperlink ref="D15" r:id="rId11" xr:uid="{397922B9-2152-478D-9B26-56C9C49440A0}"/>
+    <hyperlink ref="E7" r:id="rId12" xr:uid="{FB6E1C4C-E159-43C3-BE2F-C1EB1EE1E5EE}"/>
+    <hyperlink ref="D7" r:id="rId13" xr:uid="{A0F9795B-E883-47BB-BF86-61830DDE2952}"/>
+    <hyperlink ref="D14" r:id="rId14" xr:uid="{24CC6ADA-06BD-4669-ADD9-8DCC20582EF2}"/>
+    <hyperlink ref="E14" r:id="rId15" xr:uid="{AFD96068-6BC1-4F9B-A93D-CA39F78EFC55}"/>
+    <hyperlink ref="D19" r:id="rId16" xr:uid="{31A28E04-31A4-4E33-B54D-49645CD59584}"/>
+    <hyperlink ref="D6" r:id="rId17" xr:uid="{080A3882-7D6E-495E-972C-8B84E5F7373F}"/>
+    <hyperlink ref="C24" r:id="rId18" xr:uid="{06B9DA70-F67B-4B2D-B5FD-27CCD75C86FC}"/>
+    <hyperlink ref="D24" r:id="rId19" xr:uid="{55D11962-BE3A-40D2-A158-CC6F4E3D9FF9}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId7"/>
+  <pageSetup orientation="portrait" r:id="rId20"/>
   <tableParts count="1">
-    <tablePart r:id="rId8"/>
+    <tablePart r:id="rId21"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>